<commit_message>
feat: elearning flow for tutor and siswa including attendance, grades, and profile
</commit_message>
<xml_diff>
--- a/public/templates/DAFTAR HADIR WARGA BELAJAR PER MAPEL.xlsx
+++ b/public/templates/DAFTAR HADIR WARGA BELAJAR PER MAPEL.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Asus\Documents\E-learning\public\templates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2D6EB054-3514-462B-AFA9-197D698AEF1D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FAF8DF4B-2682-4D9D-83BB-D716AF36ED2D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -125,9 +125,6 @@
   </si>
   <si>
     <t>${table:siswa.no}</t>
-  </si>
-  <si>
-    <t>${table:siswa.nipd}</t>
   </si>
   <si>
     <t>${table:siswa.nisn}</t>
@@ -248,6 +245,9 @@
   </si>
   <si>
     <t>NO</t>
+  </si>
+  <si>
+    <t>${table:siswa.nis}</t>
   </si>
 </sst>
 </file>
@@ -473,12 +473,18 @@
     <xf numFmtId="0" fontId="10" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -500,17 +506,11 @@
     <xf numFmtId="0" fontId="9" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -883,7 +883,7 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:38" ht="15" customHeight="1">
-      <c r="A1" s="32" t="s">
+      <c r="A1" s="21" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="22"/>
@@ -925,7 +925,7 @@
       <c r="AL1" s="22"/>
     </row>
     <row r="2" spans="1:38" ht="27.75" customHeight="1">
-      <c r="A2" s="33"/>
+      <c r="A2" s="23"/>
       <c r="B2" s="22"/>
       <c r="C2" s="22"/>
       <c r="D2" s="22"/>
@@ -965,7 +965,7 @@
       <c r="AL2" s="22"/>
     </row>
     <row r="3" spans="1:38" ht="15" customHeight="1">
-      <c r="A3" s="34" t="s">
+      <c r="A3" s="24" t="s">
         <v>1</v>
       </c>
       <c r="B3" s="22"/>
@@ -1007,7 +1007,7 @@
       <c r="AL3" s="22"/>
     </row>
     <row r="4" spans="1:38" ht="15" customHeight="1">
-      <c r="A4" s="35" t="s">
+      <c r="A4" s="25" t="s">
         <v>2</v>
       </c>
       <c r="B4" s="22"/>
@@ -1049,7 +1049,7 @@
       <c r="AL4" s="22"/>
     </row>
     <row r="5" spans="1:38" ht="15" customHeight="1">
-      <c r="A5" s="35" t="s">
+      <c r="A5" s="25" t="s">
         <v>3</v>
       </c>
       <c r="B5" s="22"/>
@@ -1091,46 +1091,46 @@
       <c r="AL5" s="22"/>
     </row>
     <row r="6" spans="1:38" ht="15.75" customHeight="1">
-      <c r="A6" s="24" t="s">
+      <c r="A6" s="26" t="s">
         <v>4</v>
       </c>
-      <c r="B6" s="25"/>
-      <c r="C6" s="25"/>
-      <c r="D6" s="25"/>
-      <c r="E6" s="25"/>
-      <c r="F6" s="25"/>
-      <c r="G6" s="25"/>
-      <c r="H6" s="25"/>
-      <c r="I6" s="25"/>
-      <c r="J6" s="25"/>
-      <c r="K6" s="25"/>
-      <c r="L6" s="25"/>
-      <c r="M6" s="25"/>
-      <c r="N6" s="25"/>
-      <c r="O6" s="25"/>
-      <c r="P6" s="25"/>
-      <c r="Q6" s="25"/>
-      <c r="R6" s="25"/>
-      <c r="S6" s="25"/>
-      <c r="T6" s="25"/>
-      <c r="U6" s="25"/>
-      <c r="V6" s="25"/>
-      <c r="W6" s="25"/>
-      <c r="X6" s="25"/>
-      <c r="Y6" s="25"/>
-      <c r="Z6" s="25"/>
-      <c r="AA6" s="25"/>
-      <c r="AB6" s="25"/>
-      <c r="AC6" s="25"/>
-      <c r="AD6" s="25"/>
-      <c r="AE6" s="25"/>
-      <c r="AF6" s="25"/>
-      <c r="AG6" s="25"/>
-      <c r="AH6" s="25"/>
-      <c r="AI6" s="25"/>
-      <c r="AJ6" s="25"/>
-      <c r="AK6" s="25"/>
-      <c r="AL6" s="25"/>
+      <c r="B6" s="27"/>
+      <c r="C6" s="27"/>
+      <c r="D6" s="27"/>
+      <c r="E6" s="27"/>
+      <c r="F6" s="27"/>
+      <c r="G6" s="27"/>
+      <c r="H6" s="27"/>
+      <c r="I6" s="27"/>
+      <c r="J6" s="27"/>
+      <c r="K6" s="27"/>
+      <c r="L6" s="27"/>
+      <c r="M6" s="27"/>
+      <c r="N6" s="27"/>
+      <c r="O6" s="27"/>
+      <c r="P6" s="27"/>
+      <c r="Q6" s="27"/>
+      <c r="R6" s="27"/>
+      <c r="S6" s="27"/>
+      <c r="T6" s="27"/>
+      <c r="U6" s="27"/>
+      <c r="V6" s="27"/>
+      <c r="W6" s="27"/>
+      <c r="X6" s="27"/>
+      <c r="Y6" s="27"/>
+      <c r="Z6" s="27"/>
+      <c r="AA6" s="27"/>
+      <c r="AB6" s="27"/>
+      <c r="AC6" s="27"/>
+      <c r="AD6" s="27"/>
+      <c r="AE6" s="27"/>
+      <c r="AF6" s="27"/>
+      <c r="AG6" s="27"/>
+      <c r="AH6" s="27"/>
+      <c r="AI6" s="27"/>
+      <c r="AJ6" s="27"/>
+      <c r="AK6" s="27"/>
+      <c r="AL6" s="27"/>
     </row>
     <row r="7" spans="1:38" ht="7.5" customHeight="1">
       <c r="A7" s="1"/>
@@ -1213,7 +1213,7 @@
       <c r="AL8" s="1"/>
     </row>
     <row r="9" spans="1:38">
-      <c r="A9" s="26" t="s">
+      <c r="A9" s="28" t="s">
         <v>5</v>
       </c>
       <c r="B9" s="22"/>
@@ -1255,7 +1255,7 @@
       <c r="AL9" s="22"/>
     </row>
     <row r="10" spans="1:38">
-      <c r="A10" s="26" t="s">
+      <c r="A10" s="28" t="s">
         <v>6</v>
       </c>
       <c r="B10" s="22"/>
@@ -1297,7 +1297,7 @@
       <c r="AL10" s="22"/>
     </row>
     <row r="11" spans="1:38" ht="15.75">
-      <c r="A11" s="29" t="s">
+      <c r="A11" s="31" t="s">
         <v>7</v>
       </c>
       <c r="B11" s="22"/>
@@ -1379,7 +1379,7 @@
       <c r="AL12" s="3"/>
     </row>
     <row r="13" spans="1:38" ht="15.75">
-      <c r="A13" s="30" t="s">
+      <c r="A13" s="32" t="s">
         <v>8</v>
       </c>
       <c r="B13" s="22"/>
@@ -1515,68 +1515,68 @@
       <c r="AL15" s="3"/>
     </row>
     <row r="16" spans="1:38" ht="15.75" customHeight="1">
-      <c r="A16" s="31" t="s">
-        <v>64</v>
+      <c r="A16" s="33" t="s">
+        <v>63</v>
       </c>
-      <c r="B16" s="31" t="s">
+      <c r="B16" s="33" t="s">
         <v>16</v>
       </c>
-      <c r="C16" s="31" t="s">
+      <c r="C16" s="33" t="s">
         <v>17</v>
       </c>
-      <c r="D16" s="27" t="s">
+      <c r="D16" s="29" t="s">
         <v>18</v>
       </c>
-      <c r="E16" s="27" t="s">
+      <c r="E16" s="29" t="s">
         <v>19</v>
       </c>
-      <c r="F16" s="27" t="s">
+      <c r="F16" s="29" t="s">
         <v>20</v>
       </c>
-      <c r="G16" s="27" t="s">
+      <c r="G16" s="29" t="s">
         <v>21</v>
       </c>
-      <c r="H16" s="28"/>
-      <c r="I16" s="28"/>
-      <c r="J16" s="28"/>
-      <c r="K16" s="28"/>
-      <c r="L16" s="28"/>
-      <c r="M16" s="28"/>
-      <c r="N16" s="28"/>
-      <c r="O16" s="28"/>
-      <c r="P16" s="28"/>
-      <c r="Q16" s="28"/>
-      <c r="R16" s="28"/>
-      <c r="S16" s="28"/>
-      <c r="T16" s="28"/>
-      <c r="U16" s="28"/>
-      <c r="V16" s="28"/>
-      <c r="W16" s="28"/>
-      <c r="X16" s="28"/>
-      <c r="Y16" s="28"/>
-      <c r="Z16" s="28"/>
-      <c r="AA16" s="28"/>
-      <c r="AB16" s="28"/>
-      <c r="AC16" s="28"/>
-      <c r="AD16" s="28"/>
-      <c r="AE16" s="28"/>
-      <c r="AF16" s="28"/>
-      <c r="AG16" s="28"/>
-      <c r="AH16" s="28"/>
-      <c r="AI16" s="28"/>
-      <c r="AJ16" s="28"/>
-      <c r="AK16" s="28"/>
-      <c r="AL16" s="27" t="s">
+      <c r="H16" s="30"/>
+      <c r="I16" s="30"/>
+      <c r="J16" s="30"/>
+      <c r="K16" s="30"/>
+      <c r="L16" s="30"/>
+      <c r="M16" s="30"/>
+      <c r="N16" s="30"/>
+      <c r="O16" s="30"/>
+      <c r="P16" s="30"/>
+      <c r="Q16" s="30"/>
+      <c r="R16" s="30"/>
+      <c r="S16" s="30"/>
+      <c r="T16" s="30"/>
+      <c r="U16" s="30"/>
+      <c r="V16" s="30"/>
+      <c r="W16" s="30"/>
+      <c r="X16" s="30"/>
+      <c r="Y16" s="30"/>
+      <c r="Z16" s="30"/>
+      <c r="AA16" s="30"/>
+      <c r="AB16" s="30"/>
+      <c r="AC16" s="30"/>
+      <c r="AD16" s="30"/>
+      <c r="AE16" s="30"/>
+      <c r="AF16" s="30"/>
+      <c r="AG16" s="30"/>
+      <c r="AH16" s="30"/>
+      <c r="AI16" s="30"/>
+      <c r="AJ16" s="30"/>
+      <c r="AK16" s="30"/>
+      <c r="AL16" s="29" t="s">
         <v>22</v>
       </c>
     </row>
     <row r="17" spans="1:38" ht="28.5" customHeight="1">
-      <c r="A17" s="28"/>
-      <c r="B17" s="28"/>
-      <c r="C17" s="28"/>
-      <c r="D17" s="28"/>
-      <c r="E17" s="28"/>
-      <c r="F17" s="28"/>
+      <c r="A17" s="30"/>
+      <c r="B17" s="30"/>
+      <c r="C17" s="30"/>
+      <c r="D17" s="30"/>
+      <c r="E17" s="30"/>
+      <c r="F17" s="30"/>
       <c r="G17" s="17">
         <v>1</v>
       </c>
@@ -1670,122 +1670,122 @@
       <c r="AK17" s="17">
         <v>31</v>
       </c>
-      <c r="AL17" s="28"/>
+      <c r="AL17" s="30"/>
     </row>
     <row r="18" spans="1:38" ht="28.5" customHeight="1">
       <c r="A18" s="18" t="s">
         <v>23</v>
       </c>
       <c r="B18" s="19" t="s">
+        <v>64</v>
+      </c>
+      <c r="C18" s="19" t="s">
         <v>24</v>
       </c>
-      <c r="C18" s="19" t="s">
+      <c r="D18" s="19" t="s">
         <v>25</v>
       </c>
-      <c r="D18" s="19" t="s">
+      <c r="E18" s="19" t="s">
+        <v>62</v>
+      </c>
+      <c r="F18" s="19" t="s">
         <v>26</v>
       </c>
-      <c r="E18" s="19" t="s">
-        <v>63</v>
-      </c>
-      <c r="F18" s="19" t="s">
+      <c r="G18" s="20" t="s">
         <v>27</v>
       </c>
-      <c r="G18" s="20" t="s">
+      <c r="H18" s="20" t="s">
         <v>28</v>
       </c>
-      <c r="H18" s="20" t="s">
+      <c r="I18" s="20" t="s">
         <v>29</v>
       </c>
-      <c r="I18" s="20" t="s">
+      <c r="J18" s="20" t="s">
         <v>30</v>
       </c>
-      <c r="J18" s="20" t="s">
+      <c r="K18" s="20" t="s">
         <v>31</v>
       </c>
-      <c r="K18" s="20" t="s">
+      <c r="L18" s="20" t="s">
         <v>32</v>
       </c>
-      <c r="L18" s="20" t="s">
+      <c r="M18" s="20" t="s">
         <v>33</v>
       </c>
-      <c r="M18" s="20" t="s">
+      <c r="N18" s="20" t="s">
         <v>34</v>
       </c>
-      <c r="N18" s="20" t="s">
+      <c r="O18" s="20" t="s">
         <v>35</v>
       </c>
-      <c r="O18" s="20" t="s">
+      <c r="P18" s="20" t="s">
         <v>36</v>
       </c>
-      <c r="P18" s="20" t="s">
+      <c r="Q18" s="20" t="s">
         <v>37</v>
       </c>
-      <c r="Q18" s="20" t="s">
+      <c r="R18" s="20" t="s">
         <v>38</v>
       </c>
-      <c r="R18" s="20" t="s">
+      <c r="S18" s="20" t="s">
         <v>39</v>
       </c>
-      <c r="S18" s="20" t="s">
+      <c r="T18" s="20" t="s">
         <v>40</v>
       </c>
-      <c r="T18" s="20" t="s">
+      <c r="U18" s="20" t="s">
         <v>41</v>
       </c>
-      <c r="U18" s="20" t="s">
+      <c r="V18" s="20" t="s">
         <v>42</v>
       </c>
-      <c r="V18" s="20" t="s">
+      <c r="W18" s="20" t="s">
         <v>43</v>
       </c>
-      <c r="W18" s="20" t="s">
+      <c r="X18" s="20" t="s">
         <v>44</v>
       </c>
-      <c r="X18" s="20" t="s">
+      <c r="Y18" s="20" t="s">
         <v>45</v>
       </c>
-      <c r="Y18" s="20" t="s">
+      <c r="Z18" s="20" t="s">
         <v>46</v>
       </c>
-      <c r="Z18" s="20" t="s">
+      <c r="AA18" s="20" t="s">
         <v>47</v>
       </c>
-      <c r="AA18" s="20" t="s">
+      <c r="AB18" s="20" t="s">
         <v>48</v>
       </c>
-      <c r="AB18" s="20" t="s">
+      <c r="AC18" s="20" t="s">
         <v>49</v>
       </c>
-      <c r="AC18" s="20" t="s">
+      <c r="AD18" s="20" t="s">
         <v>50</v>
       </c>
-      <c r="AD18" s="20" t="s">
+      <c r="AE18" s="20" t="s">
         <v>51</v>
       </c>
-      <c r="AE18" s="20" t="s">
+      <c r="AF18" s="20" t="s">
         <v>52</v>
       </c>
-      <c r="AF18" s="20" t="s">
+      <c r="AG18" s="20" t="s">
         <v>53</v>
       </c>
-      <c r="AG18" s="20" t="s">
+      <c r="AH18" s="20" t="s">
         <v>54</v>
       </c>
-      <c r="AH18" s="20" t="s">
+      <c r="AI18" s="20" t="s">
         <v>55</v>
       </c>
-      <c r="AI18" s="20" t="s">
+      <c r="AJ18" s="20" t="s">
         <v>56</v>
       </c>
-      <c r="AJ18" s="20" t="s">
+      <c r="AK18" s="20" t="s">
         <v>57</v>
       </c>
-      <c r="AK18" s="20" t="s">
+      <c r="AL18" s="20" t="s">
         <v>58</v>
-      </c>
-      <c r="AL18" s="20" t="s">
-        <v>59</v>
       </c>
     </row>
     <row r="19" spans="1:38" ht="15.75" customHeight="1">
@@ -1902,8 +1902,8 @@
       <c r="AE21" s="8"/>
       <c r="AF21" s="8"/>
       <c r="AG21" s="8"/>
-      <c r="AH21" s="21" t="s">
-        <v>60</v>
+      <c r="AH21" s="34" t="s">
+        <v>59</v>
       </c>
       <c r="AI21" s="22"/>
       <c r="AJ21" s="22"/>
@@ -1984,8 +1984,8 @@
       <c r="AE23" s="8"/>
       <c r="AF23" s="8"/>
       <c r="AG23" s="8"/>
-      <c r="AH23" s="21" t="s">
-        <v>61</v>
+      <c r="AH23" s="34" t="s">
+        <v>60</v>
       </c>
       <c r="AI23" s="22"/>
       <c r="AJ23" s="22"/>
@@ -2026,7 +2026,7 @@
       <c r="AE24" s="8"/>
       <c r="AF24" s="8"/>
       <c r="AG24" s="8"/>
-      <c r="AH24" s="21"/>
+      <c r="AH24" s="34"/>
       <c r="AI24" s="22"/>
       <c r="AJ24" s="22"/>
       <c r="AK24" s="22"/>
@@ -2106,7 +2106,7 @@
       <c r="AE26" s="8"/>
       <c r="AF26" s="8"/>
       <c r="AG26" s="8"/>
-      <c r="AH26" s="23"/>
+      <c r="AH26" s="35"/>
       <c r="AI26" s="22"/>
       <c r="AJ26" s="22"/>
       <c r="AK26" s="22"/>
@@ -2146,8 +2146,8 @@
       <c r="AE27" s="8"/>
       <c r="AF27" s="8"/>
       <c r="AG27" s="8"/>
-      <c r="AH27" s="23" t="s">
-        <v>62</v>
+      <c r="AH27" s="35" t="s">
+        <v>61</v>
       </c>
       <c r="AI27" s="22"/>
       <c r="AJ27" s="22"/>
@@ -10929,11 +10929,11 @@
     <row r="1000" ht="15.75" customHeight="1"/>
   </sheetData>
   <mergeCells count="23">
-    <mergeCell ref="A1:AL1"/>
-    <mergeCell ref="A2:AL2"/>
-    <mergeCell ref="A3:AL3"/>
-    <mergeCell ref="A4:AL4"/>
-    <mergeCell ref="A5:AL5"/>
+    <mergeCell ref="AH21:AL21"/>
+    <mergeCell ref="AH23:AL23"/>
+    <mergeCell ref="AH24:AL24"/>
+    <mergeCell ref="AH26:AL26"/>
+    <mergeCell ref="AH27:AL27"/>
     <mergeCell ref="A6:AL6"/>
     <mergeCell ref="A9:AL9"/>
     <mergeCell ref="E16:E17"/>
@@ -10947,11 +10947,11 @@
     <mergeCell ref="B16:B17"/>
     <mergeCell ref="C16:C17"/>
     <mergeCell ref="D16:D17"/>
-    <mergeCell ref="AH21:AL21"/>
-    <mergeCell ref="AH23:AL23"/>
-    <mergeCell ref="AH24:AL24"/>
-    <mergeCell ref="AH26:AL26"/>
-    <mergeCell ref="AH27:AL27"/>
+    <mergeCell ref="A1:AL1"/>
+    <mergeCell ref="A2:AL2"/>
+    <mergeCell ref="A3:AL3"/>
+    <mergeCell ref="A4:AL4"/>
+    <mergeCell ref="A5:AL5"/>
   </mergeCells>
   <conditionalFormatting sqref="A18:AL18">
     <cfRule type="expression" dxfId="0" priority="1">

</xml_diff>